<commit_message>
Refactor ErrorHandling and add ErrorMeta class
</commit_message>
<xml_diff>
--- a/docs/code_plan.xlsx
+++ b/docs/code_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Box Sync\Projects\Excel_Steps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1427D5A-5FC4-4D23-981D-3B362F0735C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACBD0B5A-7556-4DF8-A5CE-7415244A6D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="495" yWindow="3285" windowWidth="28800" windowHeight="11588" xr2:uid="{A608B931-C59A-4730-A3C3-3868F80D0222}"/>
+    <workbookView xWindow="1343" yWindow="795" windowWidth="29977" windowHeight="14175" xr2:uid="{8799C181-B5A1-4CC6-B15E-D1E739BDAE9B}"/>
   </bookViews>
   <sheets>
     <sheet name="plan" sheetId="5" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Settings_" sheetId="4" state="veryHidden" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">plan!$A$1:$H$40</definedName>
     <definedName name="AfterEndorRenameColumn">ExcelSteps!$E:$E</definedName>
     <definedName name="Arguments">plan!$F:$F</definedName>
     <definedName name="Codewritinginstructions">plan!$G:$G</definedName>
@@ -62,14 +63,14 @@
     <author>j.d.landgrebe</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{6E8120FC-BF46-4AE8-9ABF-38747E5BDAE0}">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{AC51E152-EB30-435C-9361-1394993714E6}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t>Semicolon delimited</t>
         </r>
@@ -80,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="237">
   <si>
     <t>Module</t>
   </si>
@@ -352,6 +353,372 @@
     <t>Unit tests for add new key and overwrite existing key; verify object and scalar values are handled</t>
   </si>
   <si>
+    <t>ErrorHandling.cls</t>
+  </si>
+  <si>
+    <t>Error state and reporting orchestration</t>
+  </si>
+  <si>
+    <t>Init</t>
+  </si>
+  <si>
+    <t>Initialize error handling state and workbook context</t>
+  </si>
+  <si>
+    <t>wkbkE As Workbook Optional; IsHandle As Boolean Optional</t>
+  </si>
+  <si>
+    <t>Set defaults for IsHandle; code fields; ErrMsg; IsUserFacing; IsNewErr; IsShowMsgs; set wkbkE to ThisWorkbook unless argument is provided</t>
+  </si>
+  <si>
+    <t>test_Init sets defaults correctly; test wkbkE override path; test IsHandle toggle behavior</t>
+  </si>
+  <si>
+    <t>RecordErr</t>
+  </si>
+  <si>
+    <t>Record root or nested error and trigger reporting gate</t>
+  </si>
+  <si>
+    <t>Locn As String; CallingFunction As Boolean ByRef Optional</t>
+  </si>
+  <si>
+    <t>Detect driver call with IsMissing; set CallingFunction False for Boolean caller; set Locn; set iCodeReport when IsNewErr; append Called by suffix for nested non user-facing; call AppendErrMsg; report only when IsShowMsgs And IsDriverCall Or IsTesting</t>
+  </si>
+  <si>
+    <t>driver tests verify reporting gate; Boolean caller tests verify return False; nested trace tests verify Called by behavior for non user-facing</t>
+  </si>
+  <si>
+    <t>AppendErrMsg</t>
+  </si>
+  <si>
+    <t>Build and append current error message into ErrMsg</t>
+  </si>
+  <si>
+    <t>sMsgSuffix As String; Returns Boolean</t>
+  </si>
+  <si>
+    <t>For IsNewErr: call aryErrLookup; set IsUserFacing from metadata; map base marker to VBA error text; preserve existing wording for not found and developer and user-facing branches; set IsNewErr False; for nested non user-facing append suffix line</t>
+  </si>
+  <si>
+    <t>tests for not found wording; developer formatting with code and routine and ErrParam; user-facing concise branch; nested append branch</t>
+  </si>
+  <si>
+    <t>AppendErrMsg_prev</t>
+  </si>
+  <si>
+    <t>Legacy preserved version of AppendErrMsg for comparison fallback</t>
+  </si>
+  <si>
+    <t>Keep behavior aligned with current implementation until removal decision; no new call sites added</t>
+  </si>
+  <si>
+    <t>smoke test can compare output shape against AppendErrMsg for representative cases before deprecation</t>
+  </si>
+  <si>
+    <t>Error metadata lookup</t>
+  </si>
+  <si>
+    <t>aryErrLookup</t>
+  </si>
+  <si>
+    <t>Lookup Errors_ metadata row by composite report code and return metadata array</t>
+  </si>
+  <si>
+    <t>None; Returns Variant Array</t>
+  </si>
+  <si>
+    <t>Call SetTblELocations then rngMultiKeyBasic on code column; default to iErrNotFound row metadata when missing; return code; routine; message; IsUserFacing entries</t>
+  </si>
+  <si>
+    <t>tests for found row mapping; missing row fallback to Msg Not Found; base error marker behavior consumed by AppendErrMsg</t>
+  </si>
+  <si>
+    <t>Error reporting output</t>
+  </si>
+  <si>
+    <t>ReportMsg</t>
+  </si>
+  <si>
+    <t>Accumulate and optionally show current ErrMsg</t>
+  </si>
+  <si>
+    <t>None; Returns Long</t>
+  </si>
+  <si>
+    <t>Exit when IsHandle False; call UpdateMsgsAccum; if IsShowMsgs then MsgBox with Execution Error title</t>
+  </si>
+  <si>
+    <t>tests verify Msgs_accum update always when handle enabled; MsgBox path gated by IsShowMsgs</t>
+  </si>
+  <si>
+    <t>Warning and info reporting</t>
+  </si>
+  <si>
+    <t>ReportWarningMsg</t>
+  </si>
+  <si>
+    <t>Lookup and report warning or information message by local code</t>
+  </si>
+  <si>
+    <t>iCode As Integer; Locn As String; param Optional</t>
+  </si>
+  <si>
+    <t>Set Locn and iCodeLocal; call GetBaseErrCode and exit when missing; build message from aryErrLookup index 2 plus ErrParam and optional param; call UpdateMsgsAccum; gate MsgBox by IsShowMsgs; re-init errs at end</t>
+  </si>
+  <si>
+    <t>tests for warning message resolution and accumulation; missing base code exits quietly; re-init resets IsNewErr and fields</t>
+  </si>
+  <si>
+    <t>Message accumulation utilities</t>
+  </si>
+  <si>
+    <t>UpdateMsgsAccum</t>
+  </si>
+  <si>
+    <t>Append message to accumulated warnings and errors text</t>
+  </si>
+  <si>
+    <t>msg As String</t>
+  </si>
+  <si>
+    <t>Append msg and vbCrLf to Msgs_accum</t>
+  </si>
+  <si>
+    <t>tests for append order and line break behavior across multiple calls</t>
+  </si>
+  <si>
+    <t>Comment message utilities</t>
+  </si>
+  <si>
+    <t>LookupCommentMsg</t>
+  </si>
+  <si>
+    <t>Lookup a comment message and add it to a range</t>
+  </si>
+  <si>
+    <t>rng As Range; Locn As String; IsReinitialize As Boolean Optional</t>
+  </si>
+  <si>
+    <t>Set Locn; call GetBaseErrCode; if base code found add comment from aryErrLookup index 2; optionally re-init using wkbkE and IsHandle</t>
+  </si>
+  <si>
+    <t>tests for comment added on valid code; no comment when base code missing; IsReinitialize False retains state</t>
+  </si>
+  <si>
+    <t>GetBaseErrCode</t>
+  </si>
+  <si>
+    <t>Resolve base error code for current routine location</t>
+  </si>
+  <si>
+    <t>None; Returns Boolean</t>
+  </si>
+  <si>
+    <t>Locate sErrBase row using rngMultiKeyBasic against function and message columns; set iCodeBase to iErrNotFound default then overwrite when row found; return True only when found</t>
+  </si>
+  <si>
+    <t>tests for known Locn returning base code; unknown Locn returns False and iErrNotFound</t>
+  </si>
+  <si>
+    <t>SetTblELocations</t>
+  </si>
+  <si>
+    <t>Set Errors_ lookup columns and data rows range</t>
+  </si>
+  <si>
+    <t>colrngFunc ByRef; colrngMsg ByRef; colrngCode ByRef; colrngIMsg ByRef; rngRows ByRef</t>
+  </si>
+  <si>
+    <t>Use wkbkE.shtErrors columns 1;3;4;6 and last used code row to build rngRows from row 2 to last row</t>
+  </si>
+  <si>
+    <t>tests for correct column assignments; rngRows extent matches populated Errors_ table</t>
+  </si>
+  <si>
+    <t>Error state helper</t>
+  </si>
+  <si>
+    <t>IsFail</t>
+  </si>
+  <si>
+    <t>Set local error attributes when a Boolean failure condition is true</t>
+  </si>
+  <si>
+    <t>IsError As Boolean; iCode As Integer; ErrParam Optional; Returns Boolean</t>
+  </si>
+  <si>
+    <t>Return False when IsError False; when true set IsFail True; set iCodeLocal and optional ErrParam for downstream RecordErr</t>
+  </si>
+  <si>
+    <t>unit tests for true and false branches; ErrParam set only when provided</t>
+  </si>
+  <si>
+    <t>User prompt utility</t>
+  </si>
+  <si>
+    <t>ShowMessage</t>
+  </si>
+  <si>
+    <t>Lookup message and show MsgBox with configured title and text</t>
+  </si>
+  <si>
+    <t>Locn As String; iCode As Integer; vbType As Integer; param Optional; Returns Long</t>
+  </si>
+  <si>
+    <t>Default to missing base code message and title; on lookup success set iCodeLocal and message; split title and text via setMsgTitleAndText; append optional param; convert vbCrLf concat markers; return MsgBox response</t>
+  </si>
+  <si>
+    <t>tests for title split logic; default fallback path; optional param append; return value passthrough</t>
+  </si>
+  <si>
+    <t>setMsgTitleAndText</t>
+  </si>
+  <si>
+    <t>Split pipe-delimited message into title and text</t>
+  </si>
+  <si>
+    <t>sMsg As String ByRef; sTitle As String ByRef</t>
+  </si>
+  <si>
+    <t>Split on |; when only one segment set title empty and keep message; when two segments assign title first and text second</t>
+  </si>
+  <si>
+    <t>tests for one-part and two-part message strings</t>
+  </si>
+  <si>
+    <t>Warnings file lifecycle</t>
+  </si>
+  <si>
+    <t>ResetWarningsAndErrors</t>
+  </si>
+  <si>
+    <t>Reset warnings and errors setting and delete prior output file</t>
+  </si>
+  <si>
+    <t>wkbk As Workbook; sSelf As String; IsVal As Boolean Optional</t>
+  </si>
+  <si>
+    <t>Compute local path from setting; delete existing warnings file when present; initialize settings value with ParseNow and caller or Validation suffix</t>
+  </si>
+  <si>
+    <t>tests for file deletion path when file exists; settings reset format for normal and validation modes</t>
+  </si>
+  <si>
+    <t>ParseNow</t>
+  </si>
+  <si>
+    <t>Format current timestamp into fixed-length token</t>
+  </si>
+  <si>
+    <t>None; Returns String</t>
+  </si>
+  <si>
+    <t>Build YYYYMMDD_HHMM_SS string with zero padding and underscore separators</t>
+  </si>
+  <si>
+    <t>length test equals 16; format tests for separators and zero padding</t>
+  </si>
+  <si>
+    <t>WriteErrorsToFile</t>
+  </si>
+  <si>
+    <t>Write accumulated settings text to warnings and errors file and clear setting</t>
+  </si>
+  <si>
+    <t>wkbk As Workbook; IsVal As Boolean Optional</t>
+  </si>
+  <si>
+    <t>Read sSettingErrs and local path setting; fallback to ThisWorkbook.Path when missing; choose suffix _Val or datetime token; call WriteFile then DeleteSetting</t>
+  </si>
+  <si>
+    <t>tests for suffix selection in val and non-val runs; output path fallback; setting deletion after write</t>
+  </si>
+  <si>
+    <t>ErrorMeta.cls</t>
+  </si>
+  <si>
+    <t>Typed error metadata for AppendErrMsg refactor</t>
+  </si>
+  <si>
+    <t>Initialize typed metadata defaults for lookup and formatting</t>
+  </si>
+  <si>
+    <t>Set IsFound False; Code to iErrNotFound; Routine empty; Message empty; IsUserFacing False; IsBaseMessage False</t>
+  </si>
+  <si>
+    <t>test defaults after new instance</t>
+  </si>
+  <si>
+    <t>LoadFromLookup</t>
+  </si>
+  <si>
+    <t>Load one Errors_ metadata row into typed fields using current error context</t>
+  </si>
+  <si>
+    <t>errsObj As Object; Returns Boolean</t>
+  </si>
+  <si>
+    <t>Resolve report code using base plus local context; query Errors_ via existing lookup utilities; on not found set IsFound False and Message Msg Not Found then return True; on found map typed fields and set IsFound True; return False on worksheet or lookup failure</t>
+  </si>
+  <si>
+    <t>tests for found mapping; explicit not found state; missing sheet failure path</t>
+  </si>
+  <si>
+    <t>Validate</t>
+  </si>
+  <si>
+    <t>Validate loaded metadata and normalize malformed-row behavior</t>
+  </si>
+  <si>
+    <t>If IsFound False return True; validate required typed fields and boolean parseability; on malformed set Message to Malformed Errors_ Row for Locn and set malformed flag or fallback state without changing external wording contract</t>
+  </si>
+  <si>
+    <t>tests for malformed row cases including blank message and non-boolean user-facing field</t>
+  </si>
+  <si>
+    <t>ToUserMessage</t>
+  </si>
+  <si>
+    <t>Build concise user-facing message text</t>
+  </si>
+  <si>
+    <t>errParam As String; Returns String</t>
+  </si>
+  <si>
+    <t>Start from Message; append errParam when non-empty; no stack trace prefix</t>
+  </si>
+  <si>
+    <t>tests for concise output and param append</t>
+  </si>
+  <si>
+    <t>ToDeveloperMessage</t>
+  </si>
+  <si>
+    <t>Build developer-facing message text preserving legacy wording and line breaks</t>
+  </si>
+  <si>
+    <t>errCodeReport As Long; errParam As String; Returns String</t>
+  </si>
+  <si>
+    <t>Preserve existing Error code prefix and routine plus message lines; append errParam in legacy location; preserve vbCrLf behavior</t>
+  </si>
+  <si>
+    <t>tests compare output against representative legacy AppendErrMsg developer cases</t>
+  </si>
+  <si>
+    <t>Property Get and Let surface</t>
+  </si>
+  <si>
+    <t>Expose typed fields Code; Routine; Message; IsUserFacing; IsFound; IsBaseMessage for integration</t>
+  </si>
+  <si>
+    <t>Keep fields typed and avoid raw lookup array retention; ensure property setters enforce simple normalization where needed</t>
+  </si>
+  <si>
+    <t>tests for property roundtrip and default retention after initialize and clear flows</t>
+  </si>
+  <si>
     <t>Sheet</t>
   </si>
   <si>
@@ -398,6 +765,9 @@
   </si>
   <si>
     <t>Tbl_SplitCols</t>
+  </si>
+  <si>
+    <t>e</t>
   </si>
   <si>
     <t>Type</t>
@@ -461,7 +831,7 @@
       <sz val="11"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -488,7 +858,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -590,19 +960,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -644,12 +1001,12 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1007,11 +1364,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3470AA3-E873-4087-8C45-7B40D436E275}">
-  <sheetPr codeName="Sheet4">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B81E7F7A-EA8F-47F6-88CE-F9D963041001}">
+  <sheetPr codeName="Sheet4" filterMode="1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="32.59765625" style="11" customWidth="1"/>
@@ -1048,14 +1405,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:8" ht="28.5" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="20" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="12" t="s">
@@ -1074,14 +1431,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="128.25" x14ac:dyDescent="0.45">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:8" ht="128.25" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="12" t="s">
@@ -1100,14 +1457,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:8" ht="71.25" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="12" t="s">
@@ -1126,14 +1483,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:8" ht="85.5" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="12" t="s">
@@ -1152,14 +1509,14 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:8" ht="99.75" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="12" t="s">
@@ -1178,14 +1535,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:8" ht="85.5" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="12" t="s">
@@ -1204,14 +1561,14 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:8" ht="85.5" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="12" t="s">
@@ -1230,14 +1587,14 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A9" s="17" t="s">
+    <row r="9" spans="1:8" ht="71.25" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="12" t="s">
@@ -1256,14 +1613,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:8" ht="28.5" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="12" t="s">
@@ -1282,14 +1639,14 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A11" s="17" t="s">
+    <row r="11" spans="1:8" ht="71.25" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="12" t="s">
@@ -1308,14 +1665,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:8" ht="71.25" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="20" t="s">
         <v>60</v>
       </c>
       <c r="D12" s="12" t="s">
@@ -1334,14 +1691,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A13" s="17" t="s">
+    <row r="13" spans="1:8" ht="42.75" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="21" t="s">
         <v>60</v>
       </c>
       <c r="D13" s="12" t="s">
@@ -1360,14 +1717,14 @@
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:8" ht="42.75" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="21" t="s">
         <v>60</v>
       </c>
       <c r="D14" s="12" t="s">
@@ -1386,14 +1743,14 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A15" s="17" t="s">
+    <row r="15" spans="1:8" ht="42.75" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="21" t="s">
         <v>60</v>
       </c>
       <c r="D15" s="12" t="s">
@@ -1412,14 +1769,14 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A16" s="17" t="s">
+    <row r="16" spans="1:8" ht="42.75" hidden="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="21" t="s">
         <v>60</v>
       </c>
       <c r="D16" s="12" t="s">
@@ -1438,7 +1795,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:8" ht="42.75" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" s="18" t="s">
         <v>8</v>
       </c>
@@ -1464,18 +1821,624 @@
         <v>89</v>
       </c>
     </row>
+    <row r="18" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A18" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A19" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A20" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A21" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="H21" s="22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A22" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="H22" s="22" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A23" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="F23" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="H23" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="57" x14ac:dyDescent="0.45">
+      <c r="A24" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="F24" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="G24" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="H24" s="22" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A25" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="F25" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="H25" s="22" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A26" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="H26" s="22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="57" x14ac:dyDescent="0.45">
+      <c r="A27" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="F27" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="G27" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="H27" s="22" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="57" x14ac:dyDescent="0.45">
+      <c r="A28" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="E28" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="G28" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="H28" s="22" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A29" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="C29" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E29" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="G29" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="H29" s="22" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="57" x14ac:dyDescent="0.45">
+      <c r="A30" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="E30" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="F30" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="G30" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H30" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A31" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A32" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="E32" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A33" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="E33" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="F33" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="H33" s="22" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A34" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="G34" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="H34" s="22" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A35" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="F35" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="H35" s="22" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="A36" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="E36" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="G36" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="H36" s="22" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="57" x14ac:dyDescent="0.45">
+      <c r="A37" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="H37" s="22" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A38" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="F38" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="G38" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="H38" s="22" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A39" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="E39" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="F39" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="G39" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="H39" s="22" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A40" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="E40" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="F40" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="H40" s="22" t="s">
+        <v>211</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A17">
+  <autoFilter ref="A1:H40" xr:uid="{B81E7F7A-EA8F-47F6-88CE-F9D963041001}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="ErrorHandling.cls"/>
+        <filter val="ErrorMeta.cls"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="A2:A40">
     <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
       <formula>AND(SUBTOTAL(103,A1)=1, A2=A1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B17">
+  <conditionalFormatting sqref="B2:B40">
     <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
       <formula>AND(SUBTOTAL(103,B1)=1, B2=B1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C17">
+  <conditionalFormatting sqref="C2:C40">
     <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
       <formula>AND(SUBTOTAL(103,C1)=1, C2=C1)</formula>
     </cfRule>
@@ -1486,7 +2449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54337E96-5EEE-4BB1-B47D-80B867CA6903}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E5D9449-FE78-4DE2-98C2-B6D08D454C2B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1502,42 +2465,42 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>212</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>213</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>214</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>93</v>
+        <v>215</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>217</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>96</v>
+        <v>218</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>97</v>
+        <v>219</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>98</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="3"/>
@@ -1550,13 +2513,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>101</v>
+        <v>223</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="3"/>
@@ -1567,13 +2530,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="3"/>
@@ -1586,13 +2549,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>101</v>
+        <v>223</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="3"/>
@@ -1603,13 +2566,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="3"/>
@@ -1622,13 +2585,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>101</v>
+        <v>223</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="3"/>
@@ -1639,13 +2602,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="3"/>
@@ -1658,16 +2621,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -1679,21 +2642,21 @@
     </row>
     <row r="10" spans="1:9" ht="24.4" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="5" t="s">
-        <v>103</v>
+        <v>225</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="3">
@@ -1702,16 +2665,16 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -1723,16 +2686,16 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>100</v>
+        <v>222</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -1744,14 +2707,14 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
-        <v>104</v>
+        <v>226</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1761,16 +2724,16 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>105</v>
+        <v>227</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -1783,7 +2746,7 @@
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -1796,7 +2759,7 @@
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -1809,7 +2772,7 @@
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -1822,7 +2785,7 @@
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -1835,7 +2798,7 @@
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -1848,7 +2811,7 @@
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1861,7 +2824,7 @@
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -1874,7 +2837,7 @@
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -1887,7 +2850,7 @@
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -1900,7 +2863,7 @@
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -1913,7 +2876,7 @@
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="4" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -1923,22 +2886,22 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D26" s="8" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D27" s="8" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D28" s="8" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25" xr:uid="{8BB4184F-5B34-4807-BAE3-9650500A8861}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C25" xr:uid="{0552EC5C-C1FE-4E8C-A136-126BF3CAA33D}">
       <formula1>"Col_Format,Col_Insert,Col_Delete,Col_Rename,Col_AddGroup,Col_CondFormat,Col_Dropdown,Tbl_FreezeRow1,Tbl_Sort,Tbl_SplitCols,Delete_FlagRows,Delete_RowsWithVal"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1947,40 +2910,40 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADF2AECE-B3D8-4019-9C21-E478787BB72D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{116AE690-E4EA-4B96-8BE1-22A3F9712038}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>229</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>230</v>
       </c>
       <c r="C1" t="s">
-        <v>108</v>
+        <v>231</v>
       </c>
       <c r="D1" t="s">
-        <v>109</v>
+        <v>232</v>
       </c>
       <c r="E1" t="s">
-        <v>110</v>
+        <v>233</v>
       </c>
       <c r="F1" t="s">
-        <v>111</v>
+        <v>234</v>
       </c>
       <c r="G1" t="s">
-        <v>112</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>236</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>221</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -2000,7 +2963,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>236</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>

</xml_diff>